<commit_message>
ajout du paiement bitcoin phase1
</commit_message>
<xml_diff>
--- a/codes_promo.xlsx
+++ b/codes_promo.xlsx
@@ -31,7 +31,7 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>NEXUS2024</t>
+    <t>NEXUS2026</t>
   </si>
   <si>
     <t>Code ouverture société</t>
@@ -132,13 +132,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="13"/>
+        <fgColor indexed="9"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor indexed="9"/>
+        <fgColor indexed="13"/>
         <bgColor auto="1"/>
       </patternFill>
     </fill>
@@ -312,19 +312,19 @@
     <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="3" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="4" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="5" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -333,34 +333,34 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="6" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="6" fillId="3" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="10" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="13" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -537,9 +537,9 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="20000" dir="5400000">
+            <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
               <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
@@ -619,7 +619,7 @@
         </a:effectLst>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="ctr" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -646,10 +646,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -896,9 +896,9 @@
           <a:round/>
         </a:ln>
         <a:effectLst>
-          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="20000" dir="5400000">
+          <a:outerShdw sx="100000" sy="100000" kx="0" ky="0" algn="b" rotWithShape="0" blurRad="38100" dist="23000" dir="5400000">
             <a:srgbClr val="000000">
-              <a:alpha val="38000"/>
+              <a:alpha val="35000"/>
             </a:srgbClr>
           </a:outerShdw>
         </a:effectLst>
@@ -1176,7 +1176,7 @@
         <a:effectLst/>
         <a:sp3d/>
       </a:spPr>
-      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45719" tIns="45719" rIns="45719" bIns="45719" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
+      <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="overflow" horzOverflow="overflow" vert="horz" wrap="square" lIns="45718" tIns="45718" rIns="45718" bIns="45718" numCol="1" spcCol="38100" rtlCol="0" anchor="t" upright="0">
         <a:spAutoFit/>
       </a:bodyPr>
       <a:lstStyle>
@@ -1203,10 +1203,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">

</xml_diff>